<commit_message>
All The Things She Said Intro (#82): überarbeitete Show (Version 2026-10-12_1820), Take-On-Me-Fehlerplan
Stand aus dem Arbeitsverzeichnis: show.yaml, Tabelle, generierter Code und MIDI-Datei des Vorspanns,
dazu die Analyse docs/TakeOnMe-Fehlerplan.md (nur Plan, nichts umgesetzt).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/AllTheThingsSheSaidIntro_v1/quelle/struktur.xlsx
+++ b/songs/AllTheThingsSheSaidIntro_v1/quelle/struktur.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="720" yWindow="5988" windowWidth="36576" windowHeight="18600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6672" yWindow="660" windowWidth="31908" windowHeight="24192" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Struktur" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,21 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <strike val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -72,6 +87,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -528,7 +550,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="144" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>1</v>
       </c>
@@ -544,11 +566,7 @@
 Alles dunkel, der Einspieler läuft. Kurze Blinder auf die 1 von Takt 3, 4 und 5; bei Takt 6, 8 und 9,5 je ein Blinder, der über einen Takt ausklingt.</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>BLACK</t>
-        </is>
-      </c>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="6" t="n"/>
@@ -630,7 +648,7 @@
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="6" t="n"/>
     </row>
-    <row r="14" outlineLevel="1">
+    <row r="14" outlineLevel="1" ht="28.8" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>3</v>
       </c>
@@ -640,11 +658,7 @@
           <t>kurzer voller warmweißer Blinder auf allen Geräten: springt auf der 1 auf, 210 ms voll, am Ende der Viertel wieder dunkel</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>kurzer starker Blinder eine viertel</t>
-        </is>
-      </c>
+      <c r="D14" s="6" t="n"/>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="6" t="n"/>
@@ -692,11 +706,7 @@
           <t>Blinder auf der 1, gleiche Form</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>kurzer starker Blinder eine viertel</t>
-        </is>
-      </c>
+      <c r="D18" s="6" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="6" t="n"/>
@@ -744,11 +754,7 @@
           <t>Blinder auf der 1, gleiche Form</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>kurzer starker Blinder eine viertel</t>
-        </is>
-      </c>
+      <c r="D22" s="6" t="n"/>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="6" t="n"/>
@@ -786,7 +792,7 @@
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="6" t="n"/>
     </row>
-    <row r="26" outlineLevel="1">
+    <row r="26" outlineLevel="1" ht="28.8" customHeight="1">
       <c r="A26" s="4" t="n">
         <v>6</v>
       </c>
@@ -796,11 +802,7 @@
           <t>voller warmweißer Blinder auf allen Geräten auf der 1, klingt über 1 Takt aus (bis Takt 7)</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>starker Blinder fadet 1 takt lang aus</t>
-        </is>
-      </c>
+      <c r="D26" s="6" t="n"/>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="6" t="n"/>
@@ -892,11 +894,7 @@
           <t>Blinder auf der 1, klingt über 1 Takt aus (bis Takt 9)</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>starker Blinder fadet 1 takt lang aus</t>
-        </is>
-      </c>
+      <c r="D34" s="6" t="n"/>
       <c r="E34" s="5" t="n"/>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="6" t="n"/>
@@ -966,11 +964,7 @@
           <t>Blinder, klingt über 1 Takt aus (bis Takt 10,5, über die Part-Grenze hinweg)</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>starker Blinder fadet 1 takt lang aus</t>
-        </is>
-      </c>
+      <c r="D40" s="6" t="n"/>
       <c r="E40" s="5" t="n"/>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="6" t="n"/>
@@ -986,7 +980,7 @@
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="6" t="n"/>
     </row>
-    <row r="42" outlineLevel="1">
+    <row r="42" outlineLevel="1" ht="86.40000000000001" customHeight="1">
       <c r="A42" s="4" t="n">
         <v>10</v>
       </c>
@@ -1004,11 +998,7 @@
 Nur die Matrix: Lauftext "NERDS ON FIRE", einmal (fertig kurz nach Takt 14). Ab Takt 15 laufen Wasserwellen. Alle anderen Geräte sind dunkel.</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Scrolltext "NERDS ON FIRE" nur 1x</t>
-        </is>
-      </c>
+      <c r="D42" s="6" t="n"/>
       <c r="E42" s="5" t="n"/>
       <c r="F42" s="5" t="n"/>
       <c r="G42" s="6" t="n"/>
@@ -1222,7 +1212,7 @@
       <c r="F61" s="5" t="n"/>
       <c r="G61" s="6" t="n"/>
     </row>
-    <row r="62" outlineLevel="1">
+    <row r="62" outlineLevel="1" ht="28.8" customHeight="1">
       <c r="A62" s="4" t="n">
         <v>15</v>
       </c>
@@ -1232,11 +1222,7 @@
           <t>Ab hier Wasserwellen (progWaterRipple, bunte Ringe) nur auf der Matrix, tauchen über 2 Beats auf; sie laufen als Grundbild weiter bis zum Strobo</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>ab 15,00 progWaterRipple bis strobo</t>
-        </is>
-      </c>
+      <c r="D62" s="6" t="n"/>
       <c r="E62" s="5" t="n"/>
       <c r="F62" s="5" t="n"/>
       <c r="G62" s="6" t="n"/>
@@ -1318,7 +1304,7 @@
       <c r="F69" s="5" t="n"/>
       <c r="G69" s="6" t="n"/>
     </row>
-    <row r="70" outlineLevel="1">
+    <row r="70" outlineLevel="1" ht="273.6" customHeight="1">
       <c r="A70" s="4" t="n">
         <v>17</v>
       </c>
@@ -1332,18 +1318,13 @@
           <t>progBlack(18139, 15)
 matrix: progWaterRipple(18139, 15, 50, true, false)
 Ausgabe: Übergang fade 1395 ms, Blinder bei Takt 20 = 8372 ms, 2791 ms lang, Blinder blendet 0 ms ein, 140 ms voll, 2651 ms aus, Blinder bei Takt 21,5 = 12558 ms, 2791 ms lang, Blinder blendet 0 ms ein, 140 ms voll, 2651 ms aus
-Schluss (20 Beats): progBlack(13954, 20)
-   Text (Matrix): "THE NERDS ON FIRE": THE 3 x, NERDS 3 x, ON 3 x, FIRE 1 x 1395 ms, ein Durchlauf 13950 ms (über der Szene)
-      pulsiert alle 6 Beat(s), Tiefe 100 %, darunter 30 %
-   Ausgabe: Blinder bei 0 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder bei 4186 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder bei 8372 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder bei 12558 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus
-Auf der Matrix laufen die Wasserwellen weiter (der Titel-Lauftext kommt erst nach dem Sprung im Song). Blinder bei Takt 20 und 21,5, je über einen Takt ausklingend. Ab Takt 23,5 viermal im Abstand von 1,5 Takten: Blinder auf allen Geräten und ein Wort weiß über den Wellen - THE, NERDS, ON, FIRE. Alle anderen Geräte sind dunkel.</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>Scrolltext Songtitel und Interpret, 1x</t>
-        </is>
-      </c>
+Schluss (16 Beats): progBlack(11163, 20)
+   Text (Matrix): "THE NERDS ON": THE 3 x, NERDS 3 x, ON 2 x 1395 ms, ein Durchlauf 11160 ms (über Szene und Ebene, ab 0 ms bis 10814 ms, klingt 349 ms ab, pulsiert alle 6 Beat(s), Tiefe 100 %, darunter 30 %)
+   Ausgabe: Blinder bei 0 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder bei 4186 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder bei 8372 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder liegt unter dem Text
+Auf der Matrix laufen die Wasserwellen weiter (der Titel-Lauftext kommt erst nach dem Sprung im Song). Blinder bei Takt 20 und 21,5, je über einen Takt ausklingend. Ab Takt 23,5 dreimal im Abstand von 1,5 Takten: Blinder auf allen Geräten und ein Wort weiß über den Wellen - THE, NERDS, ON. Bei Takt 27,25 STOP: alles blendet in einer Achtel auf Schwarz. Alle anderen Geräte sind dunkel.</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="n"/>
       <c r="E70" s="5" t="n"/>
       <c r="F70" s="5" t="n"/>
       <c r="G70" s="6" t="n"/>
@@ -1469,7 +1450,7 @@
       <c r="F81" s="5" t="n"/>
       <c r="G81" s="6" t="n"/>
     </row>
-    <row r="82" outlineLevel="1">
+    <row r="82" outlineLevel="1" ht="28.8" customHeight="1">
       <c r="A82" s="4" t="n">
         <v>20</v>
       </c>
@@ -1479,11 +1460,7 @@
           <t>voller warmweißer Blinder auf allen Geräten auf der 1, klingt über 1 Takt aus (bis Takt 21)</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>starker Blinder fadet 1 takt lang aus</t>
-        </is>
-      </c>
+      <c r="D82" s="6" t="n"/>
       <c r="E82" s="5" t="n"/>
       <c r="F82" s="5" t="n"/>
       <c r="G82" s="6" t="n"/>
@@ -1553,11 +1530,7 @@
           <t>Blinder, klingt über 1 Takt aus (bis Takt 22,5)</t>
         </is>
       </c>
-      <c r="D88" s="6" t="inlineStr">
-        <is>
-          <t>starker Blinder fadet 1 takt lang aus</t>
-        </is>
-      </c>
+      <c r="D88" s="6" t="n"/>
       <c r="E88" s="5" t="n"/>
       <c r="F88" s="5" t="n"/>
       <c r="G88" s="6" t="n"/>
@@ -1649,11 +1622,7 @@
           <t>voller warmweißer Blinder auf allen Geräten (1,4 Sekunden), dazu "THE" weiß auf der Matrix über den Wellen: springt auf, blendet über 1,5 Takte aus</t>
         </is>
       </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>Blinder + "THE" weiß auf der Matrix, gleiche Form</t>
-        </is>
-      </c>
+      <c r="D96" s="6" t="n"/>
       <c r="E96" s="5" t="n"/>
       <c r="F96" s="5" t="n"/>
       <c r="G96" s="6" t="n"/>
@@ -1723,11 +1692,7 @@
           <t>Blinder + "NERDS" weiß auf der Matrix, gleiche Form</t>
         </is>
       </c>
-      <c r="D102" s="6" t="inlineStr">
-        <is>
-          <t>Blinder + "NERDS" weiß auf der Matrix, gleiche Form</t>
-        </is>
-      </c>
+      <c r="D102" s="6" t="n"/>
       <c r="E102" s="5" t="n"/>
       <c r="F102" s="5" t="n"/>
       <c r="G102" s="6" t="n"/>
@@ -1794,14 +1759,10 @@
       <c r="B108" s="5" t="n"/>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>Blinder + "ON" weiß auf der Matrix, gleiche Form</t>
-        </is>
-      </c>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>Blinder + "ON" weiß auf der Matrix, gleiche Form</t>
-        </is>
-      </c>
+          <t>Blinder + "ON" weiß auf der Matrix, gleiche Form (bis zum STOP bei Takt 27,25)</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="n"/>
       <c r="E108" s="5" t="n"/>
       <c r="F108" s="5" t="n"/>
       <c r="G108" s="6" t="n"/>
@@ -1828,34 +1789,71 @@
       <c r="F110" s="5" t="n"/>
       <c r="G110" s="6" t="n"/>
     </row>
-    <row r="111" outlineLevel="2">
+    <row r="111" outlineLevel="2" ht="28.8" customHeight="1">
       <c r="A111" s="4" t="n">
         <v>27.25</v>
       </c>
       <c r="B111" s="5" t="n"/>
-      <c r="C111" s="6" t="n"/>
-      <c r="D111" s="6" t="n"/>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>STOP: Wellen und "ON" auf der Matrix blenden in einer Achtel auf Schwarz; alle Geräte bleiben bis Takt 27,5 dunkel</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>STOP -&gt; alle geräte faden innerhalb von einer achtelnote auf BLACK</t>
+        </is>
+      </c>
       <c r="E111" s="5" t="n"/>
       <c r="F111" s="5" t="n"/>
       <c r="G111" s="6" t="n"/>
     </row>
-    <row r="112" outlineLevel="2">
+    <row r="112" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A112" s="4" t="n">
         <v>27.5</v>
       </c>
-      <c r="B112" s="5" t="n"/>
-      <c r="D112" s="6" t="n"/>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>strobo</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>progBlack(698, 25)
+Text (Matrix): "FIRE": steht durchgehend, ohne Pulsieren (über der Szene)
+   darunter 30 %
+Ausgabe: Blinder bei 0 ms, 698 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 349 ms aus, Blinder liegt unter dem Text
+Schluss (1 Beats): progStrobo(697, 30, 83, getRandomColor(), getRandomColor(), getRandomColor())
+   Text (Matrix): "FIRE": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+Takt 27,5: voller warmweißer Blinder auf allen Geräten (eine Viertel) und "FIRE" weiß auf der Matrix über den Wellen. Takt 27,75: Strobo in Zufallsfarben auf allen Geräten, "FIRE" schwarz ausgestanzt. Bei Takt 28 ohne Pause in den Band-Einsatz von All The Things She Said.</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="inlineStr">
+        <is>
+          <t>Blinder + "FIRE" weiß auf der Matrix, gleiche Form; bleibt danach im Strobo ausgestanzt stehen</t>
+        </is>
+      </c>
       <c r="E112" s="5" t="n"/>
       <c r="F112" s="5" t="n"/>
       <c r="G112" s="6" t="n"/>
     </row>
-    <row r="113" outlineLevel="2">
+    <row r="113" outlineLevel="2" ht="129.6" customHeight="1">
       <c r="A113" s="4" t="n">
         <v>27.75</v>
       </c>
       <c r="B113" s="5" t="n"/>
-      <c r="C113" s="6" t="n"/>
-      <c r="D113" s="6" t="n"/>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>Strobo in Zufallsfarben auf allen Geräten (eine Viertel); auf der Matrix ist "FIRE" schwarz aus dem Strobo ausgestanzt. Danach ohne Pause in den Band-Einsatz von All The Things She Said (Stern in Neon)</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="inlineStr">
+        <is>
+          <t>progStrobo(1395, 25, 83, getRandomColor(), getRandomColor(), getRandomColor())
+Text (Matrix): "FIRE": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+Strobo in Zufallsfarben auf allen Geräten; auf der Matrix ist "FIRE" schwarz aus dem Strobo ausgestanzt. Danach ohne Pause in den Band-Einsatz von All The Things She Said (Stern in Neon).</t>
+        </is>
+      </c>
       <c r="E113" s="5" t="n"/>
       <c r="F113" s="5" t="n"/>
       <c r="G113" s="6" t="n"/>
@@ -1864,15 +1862,19 @@
       <c r="A114" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B114" s="5" t="n"/>
-      <c r="C114" s="6" t="inlineStr">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Ende</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
         <is>
           <t>Blinder + "FIRE" weiß auf der Matrix, gleiche Form; bleibt danach im Strobo ausgestanzt stehen</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>Blinder + "FIRE" weiß auf der Matrix, gleiche Form</t>
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>ab hier beginnt jetzt der 1. chorus des eigentlichen songs</t>
         </is>
       </c>
       <c r="E114" s="5" t="n"/>
@@ -1884,7 +1886,7 @@
         <v>28.25</v>
       </c>
       <c r="B115" s="5" t="n"/>
-      <c r="C115" s="6" t="n"/>
+      <c r="C115" s="8" t="n"/>
       <c r="D115" s="6" t="n"/>
       <c r="E115" s="5" t="n"/>
       <c r="F115" s="5" t="n"/>
@@ -1894,12 +1896,7 @@
       <c r="A116" s="4" t="n">
         <v>28.5</v>
       </c>
-      <c r="B116" s="5" t="inlineStr">
-        <is>
-          <t>strobo</t>
-        </is>
-      </c>
-      <c r="C116" s="6" t="inlineStr">
+      <c r="C116" s="8" t="inlineStr">
         <is>
           <t>progStrobo(1395, 25, 83, getRandomColor(), getRandomColor(), getRandomColor())
 Text (Matrix): "FIRE": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
@@ -1916,7 +1913,7 @@
         <v>28.75</v>
       </c>
       <c r="B117" s="5" t="n"/>
-      <c r="C117" s="6" t="n"/>
+      <c r="C117" s="8" t="n"/>
       <c r="D117" s="6" t="n"/>
       <c r="E117" s="5" t="n"/>
       <c r="F117" s="5" t="n"/>
@@ -1926,12 +1923,7 @@
       <c r="A118" s="7" t="n">
         <v>29</v>
       </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Ende</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
+      <c r="C118" s="9" t="inlineStr">
         <is>
           <t>0 sek. BLACK</t>
         </is>
@@ -1939,5 +1931,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
songgen.py: case-Nummern fortlaufend statt in 5er-Schritten; 12 aktuelle Songs neu generiert
Frei bleiben nur case 1/2 (Lauftext am Songanfang) und die zwei Nummern hinter trailer_entry.
Damit bleiben auch lange Songs unter 127 und stehen vollständig in der MIDI-Datei.
Neu generiert (Code bis auf die Nummern gleich): ATTSS, ATTSS Intro, APT., Be Mine, Billie Jean,
Dancing On My Own, Friday I'm In Love, Girls Just Wanna Have Fun, I Love It, I Love It Intro,
I Wanna Dance With Somebody, Tell It To My Heart. I Love It Intro bekommt dabei fxBlinderUnderText
(Regel vom 10.10.2026). Abcdefu und Take On Me nicht (Tabelle/Show seit der Generierung geändert).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/AllTheThingsSheSaidIntro_v1/quelle/struktur.xlsx
+++ b/songs/AllTheThingsSheSaidIntro_v1/quelle/struktur.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>progBlack(24070, 5)
+          <t>progBlack(24070, 3)
 Ausgabe: Blinder bei Takt 3 = 4534 ms, 698 ms lang, Blinder blendet 0 ms ein, 209 ms voll, 489 ms aus, Blinder bei Takt 4 = 7325 ms, 698 ms lang, Blinder blendet 0 ms ein, 209 ms voll, 489 ms aus, Blinder bei Takt 5 = 10116 ms, 698 ms lang, Blinder blendet 0 ms ein, 209 ms voll, 489 ms aus, Blinder bei Takt 6 = 12906 ms, 2791 ms lang, Blinder blendet 0 ms ein, 140 ms voll, 2651 ms aus, Blinder bei Takt 8 = 18488 ms, 2791 ms lang, Blinder blendet 0 ms ein, 140 ms voll, 2651 ms aus, Blinder bei Takt 9,5 = 22674 ms, 2791 ms lang, Blinder blendet 0 ms ein, 140 ms voll, 2651 ms aus
 Alles dunkel, der Einspieler läuft. Kurze Blinder auf die 1 von Takt 3, 4 und 5; bei Takt 6, 8 und 9,5 je ein Blinder, der über einen Takt ausklingt.</t>
         </is>
@@ -991,8 +991,8 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>progBlack(19535, 10)
-matrix: progScrollText("NERDS ON FIRE", 19535, 90, getRandomColor(), 10)
+          <t>progBlack(19535, 4)
+matrix: progScrollText("NERDS ON FIRE", 19535, 90, getRandomColor(), 4)
 Ebene matrix: progWaterRipple (add, ab 13953 ms, baut sich 1395 ms auf)
 Ausgabe: Blinder von 'pause' klingt noch 1395 ms aus
 Nur die Matrix: Lauftext "NERDS ON FIRE", einmal (fertig kurz nach Takt 14). Ab Takt 15 laufen Wasserwellen. Alle anderen Geräte sind dunkel.</t>
@@ -1315,10 +1315,10 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>progBlack(18139, 15)
-matrix: progWaterRipple(18139, 15, 50, true, false)
+          <t>progBlack(18139, 5)
+matrix: progWaterRipple(18139, 5, 50, true, false)
 Ausgabe: Übergang fade 1395 ms, Blinder bei Takt 20 = 8372 ms, 2791 ms lang, Blinder blendet 0 ms ein, 140 ms voll, 2651 ms aus, Blinder bei Takt 21,5 = 12558 ms, 2791 ms lang, Blinder blendet 0 ms ein, 140 ms voll, 2651 ms aus
-Schluss (16 Beats): progBlack(11163, 20)
+Schluss (16 Beats): progBlack(11163, 6)
    Text (Matrix): "THE NERDS ON": THE 3 x, NERDS 3 x, ON 2 x 1395 ms, ein Durchlauf 11160 ms (über Szene und Ebene, ab 0 ms bis 10814 ms, klingt 349 ms ab, pulsiert alle 6 Beat(s), Tiefe 100 %, darunter 30 %)
    Ausgabe: Blinder bei 0 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder bei 4186 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder bei 8372 ms, 1395 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 1046 ms aus, Blinder liegt unter dem Text
 Auf der Matrix laufen die Wasserwellen weiter (der Titel-Lauftext kommt erst nach dem Sprung im Song). Blinder bei Takt 20 und 21,5, je über einen Takt ausklingend. Ab Takt 23,5 dreimal im Abstand von 1,5 Takten: Blinder auf allen Geräten und ein Wort weiß über den Wellen - THE, NERDS, ON. Bei Takt 27,25 STOP: alles blendet in einer Achtel auf Schwarz. Alle anderen Geräte sind dunkel.</t>
@@ -1819,11 +1819,11 @@
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>progBlack(698, 25)
+          <t>progBlack(698, 7)
 Text (Matrix): "FIRE": steht durchgehend, ohne Pulsieren (über der Szene)
    darunter 30 %
 Ausgabe: Blinder bei 0 ms, 698 ms lang, Blinder blendet 0 ms ein, 349 ms voll, 349 ms aus, Blinder liegt unter dem Text
-Schluss (1 Beats): progStrobo(697, 30, 83, getRandomColor(), getRandomColor(), getRandomColor())
+Schluss (1 Beats): progStrobo(697, 8, 83, getRandomColor(), getRandomColor(), getRandomColor())
    Text (Matrix): "FIRE": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
 Takt 27,5: voller warmweißer Blinder auf allen Geräten (eine Viertel) und "FIRE" weiß auf der Matrix über den Wellen. Takt 27,75: Strobo in Zufallsfarben auf allen Geräten, "FIRE" schwarz ausgestanzt. Bei Takt 28 ohne Pause in den Band-Einsatz von All The Things She Said.</t>
         </is>

</xml_diff>